<commit_message>
created metrics and first dashboard
</commit_message>
<xml_diff>
--- a/data/sample_portfolio.xlsx
+++ b/data/sample_portfolio.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a3078394ffa78545/Documents/Koolitused/2026.03.17-Andmeinseneride_täienduskoolitusprogramm/projektitoo_git/PortfolioTracker/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aleksandra\Desktop\PortfolioTracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{763F2D25-4D78-524E-B93D-02B446FD9515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601C3E6B-DE2B-4EAE-B270-88E1D27BCC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="620" windowWidth="16300" windowHeight="20400" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1770" yWindow="750" windowWidth="12120" windowHeight="13695" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="securities" sheetId="1" r:id="rId1"/>
     <sheet name="transactions" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">transactions!$A$1:$H$26</definedName>
+  </definedNames>
   <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="46">
   <si>
     <t>ticker</t>
   </si>
@@ -166,6 +169,18 @@
   </si>
   <si>
     <t>trim</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Industrials</t>
+  </si>
+  <si>
+    <t>Consumer Discretionary</t>
+  </si>
+  <si>
+    <t>Utilities</t>
   </si>
 </sst>
 </file>
@@ -358,10 +373,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -542,7 +553,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -550,7 +561,7 @@
     <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -567,7 +578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -584,7 +595,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -601,7 +612,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -618,7 +629,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -635,7 +646,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>20</v>
       </c>
@@ -648,9 +659,11 @@
       <c r="D6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="10"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E6" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>22</v>
       </c>
@@ -663,9 +676,11 @@
       <c r="D7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="10"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E7" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>24</v>
       </c>
@@ -678,9 +693,11 @@
       <c r="D8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E8" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>26</v>
       </c>
@@ -693,9 +710,11 @@
       <c r="D9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="10"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E9" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>28</v>
       </c>
@@ -708,7 +727,9 @@
       <c r="D10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="10"/>
+      <c r="E10" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -725,9 +746,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
@@ -736,7 +758,7 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -762,7 +784,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>45672</v>
       </c>
@@ -790,7 +812,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>45698</v>
       </c>
@@ -816,7 +838,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>45708</v>
       </c>
@@ -842,7 +864,7 @@
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>45721</v>
       </c>
@@ -868,7 +890,7 @@
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>45759</v>
       </c>
@@ -896,7 +918,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>45797</v>
       </c>
@@ -922,7 +944,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>45823</v>
       </c>
@@ -950,7 +972,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>45891</v>
       </c>
@@ -978,7 +1000,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>45910</v>
       </c>
@@ -1004,7 +1026,7 @@
       </c>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>45935</v>
       </c>
@@ -1030,7 +1052,7 @@
       </c>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>46037</v>
       </c>
@@ -1056,7 +1078,7 @@
       </c>
       <c r="H12" s="10"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>46042</v>
       </c>
@@ -1082,7 +1104,7 @@
       </c>
       <c r="H13" s="10"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>46046</v>
       </c>
@@ -1108,7 +1130,7 @@
       </c>
       <c r="H14" s="10"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
         <v>46050</v>
       </c>
@@ -1134,7 +1156,7 @@
       </c>
       <c r="H15" s="10"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>46053</v>
       </c>
@@ -1160,7 +1182,7 @@
       </c>
       <c r="H16" s="10"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>46057</v>
       </c>
@@ -1186,7 +1208,7 @@
       </c>
       <c r="H17" s="10"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>46060</v>
       </c>
@@ -1212,7 +1234,7 @@
       </c>
       <c r="H18" s="10"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>46098</v>
       </c>
@@ -1238,7 +1260,7 @@
       </c>
       <c r="H19" s="10"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>46102</v>
       </c>
@@ -1264,7 +1286,7 @@
       </c>
       <c r="H20" s="10"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>46107</v>
       </c>
@@ -1290,7 +1312,7 @@
       </c>
       <c r="H21" s="10"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>46113</v>
       </c>
@@ -1316,7 +1338,7 @@
       </c>
       <c r="H22" s="10"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>46128</v>
       </c>
@@ -1342,7 +1364,7 @@
       </c>
       <c r="H23" s="10"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>46145</v>
       </c>
@@ -1368,7 +1390,7 @@
       </c>
       <c r="H24" s="10"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>46167</v>
       </c>
@@ -1393,49 +1415,50 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G26" s="8"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G28" s="8"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G29" s="8"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G30" s="8"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G36" s="8"/>
     </row>
-    <row r="37" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G37" s="8"/>
     </row>
-    <row r="38" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G38" s="8"/>
     </row>
-    <row r="39" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G39" s="8"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H26" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="C2:C111" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"BUY,SELL"</formula1>

</xml_diff>